<commit_message>
Refresh live uploads and auto-reload dashboard
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -50354,7 +50354,11 @@
         <v>64682</v>
       </c>
       <c r="M330" t="inlineStr"/>
-      <c r="N330" t="inlineStr"/>
+      <c r="N330" t="inlineStr">
+        <is>
+          <t>1781971927933</t>
+        </is>
+      </c>
       <c r="O330" t="n">
         <v>0</v>
       </c>
@@ -50375,7 +50379,11 @@
         <v>0</v>
       </c>
       <c r="V330" t="inlineStr"/>
-      <c r="W330" t="inlineStr"/>
+      <c r="W330" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4719/64592/ca674f52-37b1-4a0d-a48b-c84651b8575d.jpg</t>
+        </is>
+      </c>
       <c r="X330" t="n">
         <v>0</v>
       </c>
@@ -50809,7 +50817,11 @@
         <v>64684</v>
       </c>
       <c r="M333" t="inlineStr"/>
-      <c r="N333" t="inlineStr"/>
+      <c r="N333" t="inlineStr">
+        <is>
+          <t>1781971743495</t>
+        </is>
+      </c>
       <c r="O333" t="n">
         <v>0</v>
       </c>
@@ -50830,7 +50842,11 @@
         <v>0</v>
       </c>
       <c r="V333" t="inlineStr"/>
-      <c r="W333" t="inlineStr"/>
+      <c r="W333" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4720/64594/7151839f-f186-4979-b8d3-0b19e89c5b76.jpg</t>
+        </is>
+      </c>
       <c r="X333" t="n">
         <v>0</v>
       </c>
@@ -51860,7 +51876,11 @@
         <v>151205</v>
       </c>
       <c r="M340" t="inlineStr"/>
-      <c r="N340" t="inlineStr"/>
+      <c r="N340" t="inlineStr">
+        <is>
+          <t>1781971929957</t>
+        </is>
+      </c>
       <c r="O340" t="n">
         <v>0</v>
       </c>
@@ -51881,7 +51901,11 @@
         <v>0</v>
       </c>
       <c r="V340" t="inlineStr"/>
-      <c r="W340" t="inlineStr"/>
+      <c r="W340" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4720/646492/1d9e2b82-fc01-420e-8951-c35c6cd31408.jpg</t>
+        </is>
+      </c>
       <c r="X340" t="n">
         <v>0</v>
       </c>
@@ -55240,7 +55264,11 @@
         <v>151207</v>
       </c>
       <c r="M362" t="inlineStr"/>
-      <c r="N362" t="inlineStr"/>
+      <c r="N362" t="inlineStr">
+        <is>
+          <t>1781970842335</t>
+        </is>
+      </c>
       <c r="O362" t="n">
         <v>0</v>
       </c>
@@ -55261,7 +55289,11 @@
         <v>0</v>
       </c>
       <c r="V362" t="inlineStr"/>
-      <c r="W362" t="inlineStr"/>
+      <c r="W362" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4721/646497/6e783e9c-36aa-4f09-8d51-aeaaa1873f50.jpg</t>
+        </is>
+      </c>
       <c r="X362" t="n">
         <v>0</v>
       </c>
@@ -57092,7 +57124,11 @@
         <v>64714</v>
       </c>
       <c r="M374" t="inlineStr"/>
-      <c r="N374" t="inlineStr"/>
+      <c r="N374" t="inlineStr">
+        <is>
+          <t>1781970484687</t>
+        </is>
+      </c>
       <c r="O374" t="n">
         <v>0</v>
       </c>
@@ -57113,7 +57149,11 @@
         <v>0</v>
       </c>
       <c r="V374" t="inlineStr"/>
-      <c r="W374" t="inlineStr"/>
+      <c r="W374" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4724/64624/70cd1307-d7d8-4a4d-8f5c-53964dbc4cd9.jpg</t>
+        </is>
+      </c>
       <c r="X374" t="n">
         <v>0</v>
       </c>
@@ -57241,7 +57281,11 @@
         <v>64715</v>
       </c>
       <c r="M375" t="inlineStr"/>
-      <c r="N375" t="inlineStr"/>
+      <c r="N375" t="inlineStr">
+        <is>
+          <t>1781970664668</t>
+        </is>
+      </c>
       <c r="O375" t="n">
         <v>0</v>
       </c>
@@ -57262,7 +57306,11 @@
         <v>0</v>
       </c>
       <c r="V375" t="inlineStr"/>
-      <c r="W375" t="inlineStr"/>
+      <c r="W375" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4724/64625/1df8c5ea-4859-4f83-89aa-d0c6aefc4e2a.jpg</t>
+        </is>
+      </c>
       <c r="X375" t="n">
         <v>0</v>
       </c>
@@ -59224,7 +59272,11 @@
         <v>64725</v>
       </c>
       <c r="M388" t="inlineStr"/>
-      <c r="N388" t="inlineStr"/>
+      <c r="N388" t="inlineStr">
+        <is>
+          <t>1781971564529</t>
+        </is>
+      </c>
       <c r="O388" t="n">
         <v>0</v>
       </c>
@@ -59245,7 +59297,11 @@
         <v>0</v>
       </c>
       <c r="V388" t="inlineStr"/>
-      <c r="W388" t="inlineStr"/>
+      <c r="W388" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4725/64635/54551ac3-8f0f-4845-bbd7-aa46752921ee.jpg</t>
+        </is>
+      </c>
       <c r="X388" t="n">
         <v>0</v>
       </c>
@@ -59373,7 +59429,11 @@
         <v>64726</v>
       </c>
       <c r="M389" t="inlineStr"/>
-      <c r="N389" t="inlineStr"/>
+      <c r="N389" t="inlineStr">
+        <is>
+          <t>1781971929292</t>
+        </is>
+      </c>
       <c r="O389" t="n">
         <v>0</v>
       </c>
@@ -59394,7 +59454,11 @@
         <v>0</v>
       </c>
       <c r="V389" t="inlineStr"/>
-      <c r="W389" t="inlineStr"/>
+      <c r="W389" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4725/64636/8d5b87db-edd5-421c-8864-e4b6d0ea9484.jpg</t>
+        </is>
+      </c>
       <c r="X389" t="n">
         <v>0</v>
       </c>
@@ -59522,7 +59586,11 @@
         <v>64727</v>
       </c>
       <c r="M390" t="inlineStr"/>
-      <c r="N390" t="inlineStr"/>
+      <c r="N390" t="inlineStr">
+        <is>
+          <t>1781971930377</t>
+        </is>
+      </c>
       <c r="O390" t="n">
         <v>0</v>
       </c>
@@ -59543,7 +59611,11 @@
         <v>0</v>
       </c>
       <c r="V390" t="inlineStr"/>
-      <c r="W390" t="inlineStr"/>
+      <c r="W390" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4725/64637/050779bd-644f-4a5b-b732-89dc6d56c670.jpg</t>
+        </is>
+      </c>
       <c r="X390" t="n">
         <v>0</v>
       </c>
@@ -59671,7 +59743,11 @@
         <v>64728</v>
       </c>
       <c r="M391" t="inlineStr"/>
-      <c r="N391" t="inlineStr"/>
+      <c r="N391" t="inlineStr">
+        <is>
+          <t>1781971922925</t>
+        </is>
+      </c>
       <c r="O391" t="n">
         <v>0</v>
       </c>
@@ -59692,7 +59768,11 @@
         <v>0</v>
       </c>
       <c r="V391" t="inlineStr"/>
-      <c r="W391" t="inlineStr"/>
+      <c r="W391" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4725/64638/a55339a4-2327-4cf1-9695-cc8c17e2c930.jpg</t>
+        </is>
+      </c>
       <c r="X391" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add continuous live INEC auto refresh
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -19081,7 +19081,11 @@
         <v>58525</v>
       </c>
       <c r="M123" t="inlineStr"/>
-      <c r="N123" t="inlineStr"/>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>1781973209406</t>
+        </is>
+      </c>
       <c r="O123" t="n">
         <v>0</v>
       </c>
@@ -19102,7 +19106,11 @@
         <v>0</v>
       </c>
       <c r="V123" t="inlineStr"/>
-      <c r="W123" t="inlineStr"/>
+      <c r="W123" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4348/58434/c69a8fdf-0591-46d7-8d9a-b52a91152a60.jpg</t>
+        </is>
+      </c>
       <c r="X123" t="n">
         <v>0</v>
       </c>
@@ -42959,7 +42967,11 @@
         <v>148718</v>
       </c>
       <c r="M281" t="inlineStr"/>
-      <c r="N281" t="inlineStr"/>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>1781973016521</t>
+        </is>
+      </c>
       <c r="O281" t="n">
         <v>0</v>
       </c>
@@ -42980,7 +42992,11 @@
         <v>0</v>
       </c>
       <c r="V281" t="inlineStr"/>
-      <c r="W281" t="inlineStr"/>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4356/644006/e9c83f38-18b2-4c30-a3a0-7bb10ffd1510.jpg</t>
+        </is>
+      </c>
       <c r="X281" t="n">
         <v>0</v>
       </c>
@@ -50205,7 +50221,11 @@
         <v>64681</v>
       </c>
       <c r="M329" t="inlineStr"/>
-      <c r="N329" t="inlineStr"/>
+      <c r="N329" t="inlineStr">
+        <is>
+          <t>1781972104104</t>
+        </is>
+      </c>
       <c r="O329" t="n">
         <v>0</v>
       </c>
@@ -50226,7 +50246,11 @@
         <v>0</v>
       </c>
       <c r="V329" t="inlineStr"/>
-      <c r="W329" t="inlineStr"/>
+      <c r="W329" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4719/64591/670ec5c9-117c-4b27-a33c-ffde65397f76.jpg</t>
+        </is>
+      </c>
       <c r="X329" t="n">
         <v>0</v>
       </c>
@@ -50974,7 +50998,11 @@
         <v>64685</v>
       </c>
       <c r="M334" t="inlineStr"/>
-      <c r="N334" t="inlineStr"/>
+      <c r="N334" t="inlineStr">
+        <is>
+          <t>1781973205953</t>
+        </is>
+      </c>
       <c r="O334" t="n">
         <v>0</v>
       </c>
@@ -50995,7 +51023,11 @@
         <v>0</v>
       </c>
       <c r="V334" t="inlineStr"/>
-      <c r="W334" t="inlineStr"/>
+      <c r="W334" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4720/64595/77179fd6-3eef-45c9-be42-c08e55b27d40.jpg</t>
+        </is>
+      </c>
       <c r="X334" t="n">
         <v>0</v>
       </c>
@@ -51272,7 +51304,11 @@
         <v>64687</v>
       </c>
       <c r="M336" t="inlineStr"/>
-      <c r="N336" t="inlineStr"/>
+      <c r="N336" t="inlineStr">
+        <is>
+          <t>1781973382923</t>
+        </is>
+      </c>
       <c r="O336" t="n">
         <v>0</v>
       </c>
@@ -51293,7 +51329,11 @@
         <v>0</v>
       </c>
       <c r="V336" t="inlineStr"/>
-      <c r="W336" t="inlineStr"/>
+      <c r="W336" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4720/64597/6e3e07b3-6877-4111-9684-0d8acbf7a470.jpg</t>
+        </is>
+      </c>
       <c r="X336" t="n">
         <v>0</v>
       </c>
@@ -52182,7 +52222,11 @@
         <v>64705</v>
       </c>
       <c r="M342" t="inlineStr"/>
-      <c r="N342" t="inlineStr"/>
+      <c r="N342" t="inlineStr">
+        <is>
+          <t>1781972103673</t>
+        </is>
+      </c>
       <c r="O342" t="n">
         <v>0</v>
       </c>
@@ -52203,7 +52247,11 @@
         <v>0</v>
       </c>
       <c r="V342" t="inlineStr"/>
-      <c r="W342" t="inlineStr"/>
+      <c r="W342" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4723/64615/a95a9781-55cf-4f3c-8ad0-e3cf04378620.jpg</t>
+        </is>
+      </c>
       <c r="X342" t="n">
         <v>0</v>
       </c>
@@ -52488,7 +52536,11 @@
         <v>64707</v>
       </c>
       <c r="M344" t="inlineStr"/>
-      <c r="N344" t="inlineStr"/>
+      <c r="N344" t="inlineStr">
+        <is>
+          <t>1781972285799</t>
+        </is>
+      </c>
       <c r="O344" t="n">
         <v>0</v>
       </c>
@@ -52509,7 +52561,11 @@
         <v>0</v>
       </c>
       <c r="V344" t="inlineStr"/>
-      <c r="W344" t="inlineStr"/>
+      <c r="W344" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4723/64617/c4f5d63c-4af7-48dd-98ed-0a67c76ecc76.jpg</t>
+        </is>
+      </c>
       <c r="X344" t="n">
         <v>0</v>
       </c>
@@ -52637,7 +52693,11 @@
         <v>64708</v>
       </c>
       <c r="M345" t="inlineStr"/>
-      <c r="N345" t="inlineStr"/>
+      <c r="N345" t="inlineStr">
+        <is>
+          <t>1781972289321</t>
+        </is>
+      </c>
       <c r="O345" t="n">
         <v>0</v>
       </c>
@@ -52658,7 +52718,11 @@
         <v>0</v>
       </c>
       <c r="V345" t="inlineStr"/>
-      <c r="W345" t="inlineStr"/>
+      <c r="W345" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4723/64618/72ad9035-c4c4-4006-b9f3-c20edc91c97d.jpg</t>
+        </is>
+      </c>
       <c r="X345" t="n">
         <v>0</v>
       </c>
@@ -52786,7 +52850,11 @@
         <v>64709</v>
       </c>
       <c r="M346" t="inlineStr"/>
-      <c r="N346" t="inlineStr"/>
+      <c r="N346" t="inlineStr">
+        <is>
+          <t>1781972469858</t>
+        </is>
+      </c>
       <c r="O346" t="n">
         <v>0</v>
       </c>
@@ -52807,7 +52875,11 @@
         <v>0</v>
       </c>
       <c r="V346" t="inlineStr"/>
-      <c r="W346" t="inlineStr"/>
+      <c r="W346" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4723/64619/702b3d56-62d9-4b66-8caa-7149c05e2b6f.jpg</t>
+        </is>
+      </c>
       <c r="X346" t="n">
         <v>0</v>
       </c>
@@ -52935,7 +53007,11 @@
         <v>64710</v>
       </c>
       <c r="M347" t="inlineStr"/>
-      <c r="N347" t="inlineStr"/>
+      <c r="N347" t="inlineStr">
+        <is>
+          <t>1781972471092</t>
+        </is>
+      </c>
       <c r="O347" t="n">
         <v>0</v>
       </c>
@@ -52956,7 +53032,11 @@
         <v>0</v>
       </c>
       <c r="V347" t="inlineStr"/>
-      <c r="W347" t="inlineStr"/>
+      <c r="W347" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4723/64620/6e2896ac-f65d-4d7d-a102-587a87a3a1a6.jpg</t>
+        </is>
+      </c>
       <c r="X347" t="n">
         <v>0</v>
       </c>
@@ -53547,7 +53627,11 @@
         <v>151212</v>
       </c>
       <c r="M351" t="inlineStr"/>
-      <c r="N351" t="inlineStr"/>
+      <c r="N351" t="inlineStr">
+        <is>
+          <t>1781972468063</t>
+        </is>
+      </c>
       <c r="O351" t="n">
         <v>0</v>
       </c>
@@ -53568,7 +53652,11 @@
         <v>0</v>
       </c>
       <c r="V351" t="inlineStr"/>
-      <c r="W351" t="inlineStr"/>
+      <c r="W351" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4723/646494/97490551-aec4-4954-b67f-4d425ac1863f.jpg</t>
+        </is>
+      </c>
       <c r="X351" t="n">
         <v>0</v>
       </c>
@@ -56504,7 +56592,11 @@
         <v>64703</v>
       </c>
       <c r="M370" t="inlineStr"/>
-      <c r="N370" t="inlineStr"/>
+      <c r="N370" t="inlineStr">
+        <is>
+          <t>1781972284783</t>
+        </is>
+      </c>
       <c r="O370" t="n">
         <v>0</v>
       </c>
@@ -56525,7 +56617,11 @@
         <v>0</v>
       </c>
       <c r="V370" t="inlineStr"/>
-      <c r="W370" t="inlineStr"/>
+      <c r="W370" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4722/64613/bbf2dd97-9e62-4b41-a7bb-d2e629535220.jpg</t>
+        </is>
+      </c>
       <c r="X370" t="n">
         <v>0</v>
       </c>
@@ -60057,7 +60153,11 @@
         <v>151218</v>
       </c>
       <c r="M393" t="inlineStr"/>
-      <c r="N393" t="inlineStr"/>
+      <c r="N393" t="inlineStr">
+        <is>
+          <t>1781972103434</t>
+        </is>
+      </c>
       <c r="O393" t="n">
         <v>0</v>
       </c>
@@ -60078,7 +60178,11 @@
         <v>0</v>
       </c>
       <c r="V393" t="inlineStr"/>
-      <c r="W393" t="inlineStr"/>
+      <c r="W393" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4725/646505/cf6c98ff-500f-45ec-8dd2-01115ab808d2.jpg</t>
+        </is>
+      </c>
       <c r="X393" t="n">
         <v>0</v>
       </c>
@@ -60206,7 +60310,11 @@
         <v>151219</v>
       </c>
       <c r="M394" t="inlineStr"/>
-      <c r="N394" t="inlineStr"/>
+      <c r="N394" t="inlineStr">
+        <is>
+          <t>1781972285399</t>
+        </is>
+      </c>
       <c r="O394" t="n">
         <v>0</v>
       </c>
@@ -60227,7 +60335,11 @@
         <v>0</v>
       </c>
       <c r="V394" t="inlineStr"/>
-      <c r="W394" t="inlineStr"/>
+      <c r="W394" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4725/646506/3aab3f6c-045d-4151-b266-7cbecfe080e9.jpg</t>
+        </is>
+      </c>
       <c r="X394" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 11:43:15
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -15912,7 +15912,11 @@
         <v>148654</v>
       </c>
       <c r="M102" t="inlineStr"/>
-      <c r="N102" t="inlineStr"/>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>1781973550353</t>
+        </is>
+      </c>
       <c r="O102" t="n">
         <v>0</v>
       </c>
@@ -15933,7 +15937,11 @@
         <v>0</v>
       </c>
       <c r="V102" t="inlineStr"/>
-      <c r="W102" t="inlineStr"/>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4347/643942/2a4e5e43-3748-437a-b574-3f8acbff9286.jpg</t>
+        </is>
+      </c>
       <c r="X102" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 11:48:25
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -2977,7 +2977,11 @@
         <v>58451</v>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>1781973555290</t>
+        </is>
+      </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
@@ -2998,7 +3002,11 @@
         <v>0</v>
       </c>
       <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58360/dfb4289b-fed2-4527-82f5-8a8049feec61.jpg</t>
+        </is>
+      </c>
       <c r="X17" t="n">
         <v>0</v>
       </c>
@@ -4185,7 +4193,11 @@
         <v>58455</v>
       </c>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>1781973742525</t>
+        </is>
+      </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
@@ -4206,7 +4218,11 @@
         <v>0</v>
       </c>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4345/58364/07dc3aae-4511-4e1b-bc4b-a2d2c46da04d.jpg</t>
+        </is>
+      </c>
       <c r="X25" t="n">
         <v>0</v>
       </c>
@@ -25129,7 +25145,11 @@
         <v>58553</v>
       </c>
       <c r="M163" t="inlineStr"/>
-      <c r="N163" t="inlineStr"/>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>1781973544939</t>
+        </is>
+      </c>
       <c r="O163" t="n">
         <v>0</v>
       </c>
@@ -25150,7 +25170,11 @@
         <v>0</v>
       </c>
       <c r="V163" t="inlineStr"/>
-      <c r="W163" t="inlineStr"/>
+      <c r="W163" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4350/58462/6516dd45-5c16-4956-95f2-48cc71f0555e.jpg</t>
+        </is>
+      </c>
       <c r="X163" t="n">
         <v>0</v>
       </c>
@@ -27686,7 +27710,11 @@
         <v>148683</v>
       </c>
       <c r="M180" t="inlineStr"/>
-      <c r="N180" t="inlineStr"/>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>1781973740358</t>
+        </is>
+      </c>
       <c r="O180" t="n">
         <v>0</v>
       </c>
@@ -27707,7 +27735,11 @@
         <v>0</v>
       </c>
       <c r="V180" t="inlineStr"/>
-      <c r="W180" t="inlineStr"/>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4351/643971/f52dc953-a60a-4665-8b4f-ac5504de9041.jpg</t>
+        </is>
+      </c>
       <c r="X180" t="n">
         <v>0</v>
       </c>
@@ -35860,7 +35892,11 @@
         <v>58598</v>
       </c>
       <c r="M234" t="inlineStr"/>
-      <c r="N234" t="inlineStr"/>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>1781973688827</t>
+        </is>
+      </c>
       <c r="O234" t="n">
         <v>0</v>
       </c>
@@ -35881,7 +35917,11 @@
         <v>0</v>
       </c>
       <c r="V234" t="inlineStr"/>
-      <c r="W234" t="inlineStr"/>
+      <c r="W234" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4353/58507/019d3f5c-3480-4540-bbd6-aa017e110586.jpg</t>
+        </is>
+      </c>
       <c r="X234" t="n">
         <v>0</v>
       </c>
@@ -49029,7 +49069,11 @@
         <v>64674</v>
       </c>
       <c r="M321" t="inlineStr"/>
-      <c r="N321" t="inlineStr"/>
+      <c r="N321" t="inlineStr">
+        <is>
+          <t>1781973933925</t>
+        </is>
+      </c>
       <c r="O321" t="n">
         <v>0</v>
       </c>
@@ -49050,7 +49094,11 @@
         <v>0</v>
       </c>
       <c r="V321" t="inlineStr"/>
-      <c r="W321" t="inlineStr"/>
+      <c r="W321" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4718/64584/fbd03aa7-e746-4070-9129-9979e84d8036.jpg</t>
+        </is>
+      </c>
       <c r="X321" t="n">
         <v>0</v>
       </c>
@@ -58309,7 +58357,11 @@
         <v>64721</v>
       </c>
       <c r="M381" t="inlineStr"/>
-      <c r="N381" t="inlineStr"/>
+      <c r="N381" t="inlineStr">
+        <is>
+          <t>1781973924024</t>
+        </is>
+      </c>
       <c r="O381" t="n">
         <v>0</v>
       </c>
@@ -58330,7 +58382,11 @@
         <v>0</v>
       </c>
       <c r="V381" t="inlineStr"/>
-      <c r="W381" t="inlineStr"/>
+      <c r="W381" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4724/64631/7fd4d2b1-fc11-41e9-b238-faacf20264bc.jpg</t>
+        </is>
+      </c>
       <c r="X381" t="n">
         <v>0</v>
       </c>
@@ -58607,7 +58663,11 @@
         <v>151216</v>
       </c>
       <c r="M383" t="inlineStr"/>
-      <c r="N383" t="inlineStr"/>
+      <c r="N383" t="inlineStr">
+        <is>
+          <t>1781973731518</t>
+        </is>
+      </c>
       <c r="O383" t="n">
         <v>0</v>
       </c>
@@ -58628,7 +58688,11 @@
         <v>0</v>
       </c>
       <c r="V383" t="inlineStr"/>
-      <c r="W383" t="inlineStr"/>
+      <c r="W383" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4724/646503/2b611837-2b29-42a8-9058-9e3d68f8b5c9.jpg</t>
+        </is>
+      </c>
       <c r="X383" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 12:02:28
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -1471,7 +1471,11 @@
         <v>58441</v>
       </c>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1781974451377</t>
+        </is>
+      </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
@@ -1492,7 +1496,11 @@
         <v>0</v>
       </c>
       <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58350/d5bbb9f7-bf7a-4f30-a5b6-d6d7de510331.jpg</t>
+        </is>
+      </c>
       <c r="X7" t="n">
         <v>0</v>
       </c>
@@ -23325,7 +23333,11 @@
         <v>148670</v>
       </c>
       <c r="M151" t="inlineStr"/>
-      <c r="N151" t="inlineStr"/>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>1781974451315</t>
+        </is>
+      </c>
       <c r="O151" t="n">
         <v>0</v>
       </c>
@@ -23346,7 +23358,11 @@
         <v>0</v>
       </c>
       <c r="V151" t="inlineStr"/>
-      <c r="W151" t="inlineStr"/>
+      <c r="W151" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4349/643958/6130b112-dc31-41a9-b171-8fd096b2248d.jpg</t>
+        </is>
+      </c>
       <c r="X151" t="n">
         <v>0</v>
       </c>
@@ -26510,7 +26526,11 @@
         <v>58558</v>
       </c>
       <c r="M172" t="inlineStr"/>
-      <c r="N172" t="inlineStr"/>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>1781974092751</t>
+        </is>
+      </c>
       <c r="O172" t="n">
         <v>0</v>
       </c>
@@ -26531,7 +26551,11 @@
         <v>0</v>
       </c>
       <c r="V172" t="inlineStr"/>
-      <c r="W172" t="inlineStr"/>
+      <c r="W172" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4351/58467/22cd83d3-7440-4eff-8f98-5199a445c291.jpg</t>
+        </is>
+      </c>
       <c r="X172" t="n">
         <v>0</v>
       </c>
@@ -27561,7 +27585,11 @@
         <v>148682</v>
       </c>
       <c r="M179" t="inlineStr"/>
-      <c r="N179" t="inlineStr"/>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>1781974631552</t>
+        </is>
+      </c>
       <c r="O179" t="n">
         <v>0</v>
       </c>
@@ -27582,7 +27610,11 @@
         <v>0</v>
       </c>
       <c r="V179" t="inlineStr"/>
-      <c r="W179" t="inlineStr"/>
+      <c r="W179" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4351/643970/214f0553-0675-44f0-963d-055e7c52a63d.jpg</t>
+        </is>
+      </c>
       <c r="X179" t="n">
         <v>0</v>
       </c>
@@ -38944,7 +38976,11 @@
         <v>58607</v>
       </c>
       <c r="M254" t="inlineStr"/>
-      <c r="N254" t="inlineStr"/>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>1781974805143</t>
+        </is>
+      </c>
       <c r="O254" t="n">
         <v>0</v>
       </c>
@@ -38965,7 +39001,11 @@
         <v>0</v>
       </c>
       <c r="V254" t="inlineStr"/>
-      <c r="W254" t="inlineStr"/>
+      <c r="W254" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4354/58516/ba1c4c1b-329b-446b-9bba-396a3b8c3d4f.jpg</t>
+        </is>
+      </c>
       <c r="X254" t="n">
         <v>0</v>
       </c>
@@ -39093,7 +39133,11 @@
         <v>58608</v>
       </c>
       <c r="M255" t="inlineStr"/>
-      <c r="N255" t="inlineStr"/>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>1781974803716</t>
+        </is>
+      </c>
       <c r="O255" t="n">
         <v>0</v>
       </c>
@@ -39114,7 +39158,11 @@
         <v>0</v>
       </c>
       <c r="V255" t="inlineStr"/>
-      <c r="W255" t="inlineStr"/>
+      <c r="W255" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4354/58517/752e7012-8340-4c9c-b586-da3c73ab7726.jpg</t>
+        </is>
+      </c>
       <c r="X255" t="n">
         <v>0</v>
       </c>
@@ -49226,7 +49274,11 @@
         <v>64675</v>
       </c>
       <c r="M322" t="inlineStr"/>
-      <c r="N322" t="inlineStr"/>
+      <c r="N322" t="inlineStr">
+        <is>
+          <t>1781974088014</t>
+        </is>
+      </c>
       <c r="O322" t="n">
         <v>0</v>
       </c>
@@ -49247,7 +49299,11 @@
         <v>0</v>
       </c>
       <c r="V322" t="inlineStr"/>
-      <c r="W322" t="inlineStr"/>
+      <c r="W322" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4718/64585/a945ae17-2808-43c2-9cdf-a1c4b0a8d324.jpg</t>
+        </is>
+      </c>
       <c r="X322" t="n">
         <v>0</v>
       </c>
@@ -49532,7 +49588,11 @@
         <v>64677</v>
       </c>
       <c r="M324" t="inlineStr"/>
-      <c r="N324" t="inlineStr"/>
+      <c r="N324" t="inlineStr">
+        <is>
+          <t>1781974092259</t>
+        </is>
+      </c>
       <c r="O324" t="n">
         <v>0</v>
       </c>
@@ -49553,7 +49613,11 @@
         <v>0</v>
       </c>
       <c r="V324" t="inlineStr"/>
-      <c r="W324" t="inlineStr"/>
+      <c r="W324" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4718/64587/0f0d7aeb-6fa7-4ec3-b731-baa5a9d40487.jpg</t>
+        </is>
+      </c>
       <c r="X324" t="n">
         <v>0</v>
       </c>
@@ -49830,7 +49894,11 @@
         <v>64678</v>
       </c>
       <c r="M326" t="inlineStr"/>
-      <c r="N326" t="inlineStr"/>
+      <c r="N326" t="inlineStr">
+        <is>
+          <t>1781974089761</t>
+        </is>
+      </c>
       <c r="O326" t="n">
         <v>0</v>
       </c>
@@ -49851,7 +49919,11 @@
         <v>0</v>
       </c>
       <c r="V326" t="inlineStr"/>
-      <c r="W326" t="inlineStr"/>
+      <c r="W326" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4719/64588/c2c618f2-0954-4fdd-8536-ac0a30f707bb.jpg</t>
+        </is>
+      </c>
       <c r="X326" t="n">
         <v>0</v>
       </c>
@@ -53220,7 +53292,11 @@
         <v>64711</v>
       </c>
       <c r="M348" t="inlineStr"/>
-      <c r="N348" t="inlineStr"/>
+      <c r="N348" t="inlineStr">
+        <is>
+          <t>1781974265481</t>
+        </is>
+      </c>
       <c r="O348" t="n">
         <v>0</v>
       </c>
@@ -53241,7 +53317,11 @@
         <v>0</v>
       </c>
       <c r="V348" t="inlineStr"/>
-      <c r="W348" t="inlineStr"/>
+      <c r="W348" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4723/64621/52b5bd03-f9e0-4a4b-9de9-0646ebcf0d33.jpg</t>
+        </is>
+      </c>
       <c r="X348" t="n">
         <v>0</v>
       </c>
@@ -53840,7 +53920,11 @@
         <v>151213</v>
       </c>
       <c r="M352" t="inlineStr"/>
-      <c r="N352" t="inlineStr"/>
+      <c r="N352" t="inlineStr">
+        <is>
+          <t>1781974266632</t>
+        </is>
+      </c>
       <c r="O352" t="n">
         <v>0</v>
       </c>
@@ -53861,7 +53945,11 @@
         <v>0</v>
       </c>
       <c r="V352" t="inlineStr"/>
-      <c r="W352" t="inlineStr"/>
+      <c r="W352" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4723/646495/60f2105a-f6c5-424f-8e6e-a69b8585efe3.jpg</t>
+        </is>
+      </c>
       <c r="X352" t="n">
         <v>0</v>
       </c>
@@ -64594,7 +64682,11 @@
         <v>64754</v>
       </c>
       <c r="M422" t="inlineStr"/>
-      <c r="N422" t="inlineStr"/>
+      <c r="N422" t="inlineStr">
+        <is>
+          <t>1781974086141</t>
+        </is>
+      </c>
       <c r="O422" t="n">
         <v>0</v>
       </c>
@@ -64615,7 +64707,11 @@
         <v>0</v>
       </c>
       <c r="V422" t="inlineStr"/>
-      <c r="W422" t="inlineStr"/>
+      <c r="W422" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4728/64664/1c93ce1b-22f4-4579-b53e-9aa04552bd31.jpg</t>
+        </is>
+      </c>
       <c r="X422" t="n">
         <v>0</v>
       </c>
@@ -67181,7 +67277,11 @@
         <v>64765</v>
       </c>
       <c r="M439" t="inlineStr"/>
-      <c r="N439" t="inlineStr"/>
+      <c r="N439" t="inlineStr">
+        <is>
+          <t>1781974266039</t>
+        </is>
+      </c>
       <c r="O439" t="n">
         <v>0</v>
       </c>
@@ -67202,7 +67302,11 @@
         <v>0</v>
       </c>
       <c r="V439" t="inlineStr"/>
-      <c r="W439" t="inlineStr"/>
+      <c r="W439" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4730/64675/c080c04b-3dcf-4f18-a636-9c1e29e33e9b.jpg</t>
+        </is>
+      </c>
       <c r="X439" t="n">
         <v>0</v>
       </c>
@@ -67636,7 +67740,11 @@
         <v>64768</v>
       </c>
       <c r="M442" t="inlineStr"/>
-      <c r="N442" t="inlineStr"/>
+      <c r="N442" t="inlineStr">
+        <is>
+          <t>1781974266070</t>
+        </is>
+      </c>
       <c r="O442" t="n">
         <v>0</v>
       </c>
@@ -67657,7 +67765,11 @@
         <v>0</v>
       </c>
       <c r="V442" t="inlineStr"/>
-      <c r="W442" t="inlineStr"/>
+      <c r="W442" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4730/64678/57a0b365-235c-46f5-8e1d-7a6785359c5e.jpg</t>
+        </is>
+      </c>
       <c r="X442" t="n">
         <v>0</v>
       </c>
@@ -67785,7 +67897,11 @@
         <v>64769</v>
       </c>
       <c r="M443" t="inlineStr"/>
-      <c r="N443" t="inlineStr"/>
+      <c r="N443" t="inlineStr">
+        <is>
+          <t>1781974447124</t>
+        </is>
+      </c>
       <c r="O443" t="n">
         <v>0</v>
       </c>
@@ -67806,7 +67922,11 @@
         <v>0</v>
       </c>
       <c r="V443" t="inlineStr"/>
-      <c r="W443" t="inlineStr"/>
+      <c r="W443" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4730/64679/5b0e1ed0-9516-410b-8420-efafdc8a4266.jpg</t>
+        </is>
+      </c>
       <c r="X443" t="n">
         <v>0</v>
       </c>
@@ -67934,7 +68054,11 @@
         <v>64770</v>
       </c>
       <c r="M444" t="inlineStr"/>
-      <c r="N444" t="inlineStr"/>
+      <c r="N444" t="inlineStr">
+        <is>
+          <t>1781974628327</t>
+        </is>
+      </c>
       <c r="O444" t="n">
         <v>0</v>
       </c>
@@ -67955,7 +68079,11 @@
         <v>0</v>
       </c>
       <c r="V444" t="inlineStr"/>
-      <c r="W444" t="inlineStr"/>
+      <c r="W444" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4730/64680/fdf8717e-7fdf-4759-bdf4-67bcd20030a1.jpg</t>
+        </is>
+      </c>
       <c r="X444" t="n">
         <v>0</v>
       </c>
@@ -68083,7 +68211,11 @@
         <v>64771</v>
       </c>
       <c r="M445" t="inlineStr"/>
-      <c r="N445" t="inlineStr"/>
+      <c r="N445" t="inlineStr">
+        <is>
+          <t>1781974630372</t>
+        </is>
+      </c>
       <c r="O445" t="n">
         <v>0</v>
       </c>
@@ -68104,7 +68236,11 @@
         <v>0</v>
       </c>
       <c r="V445" t="inlineStr"/>
-      <c r="W445" t="inlineStr"/>
+      <c r="W445" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4730/64681/47783bab-a75e-4ab2-a6d9-c154eca2e745.jpg</t>
+        </is>
+      </c>
       <c r="X445" t="n">
         <v>0</v>
       </c>
@@ -68389,7 +68525,11 @@
         <v>151229</v>
       </c>
       <c r="M447" t="inlineStr"/>
-      <c r="N447" t="inlineStr"/>
+      <c r="N447" t="inlineStr">
+        <is>
+          <t>1781974627113</t>
+        </is>
+      </c>
       <c r="O447" t="n">
         <v>0</v>
       </c>
@@ -68410,7 +68550,11 @@
         <v>0</v>
       </c>
       <c r="V447" t="inlineStr"/>
-      <c r="W447" t="inlineStr"/>
+      <c r="W447" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4730/646516/066acd00-5fa0-4076-909b-7e86563f62e7.jpg</t>
+        </is>
+      </c>
       <c r="X447" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 12:16:01
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -1628,7 +1628,11 @@
         <v>58442</v>
       </c>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1781974805896</t>
+        </is>
+      </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
@@ -1649,7 +1653,11 @@
         <v>0</v>
       </c>
       <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58351/c483a830-4a28-481d-8f58-8b2bac7ec44a.jpg</t>
+        </is>
+      </c>
       <c r="X8" t="n">
         <v>0</v>
       </c>
@@ -2224,7 +2232,11 @@
         <v>58446</v>
       </c>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>1781974804121</t>
+        </is>
+      </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
@@ -2245,7 +2257,11 @@
         <v>0</v>
       </c>
       <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58355/dc5b9bbd-7012-43f1-8097-0c3026645583.jpg</t>
+        </is>
+      </c>
       <c r="X12" t="n">
         <v>0</v>
       </c>
@@ -39290,7 +39306,11 @@
         <v>58609</v>
       </c>
       <c r="M256" t="inlineStr"/>
-      <c r="N256" t="inlineStr"/>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>1781974985362</t>
+        </is>
+      </c>
       <c r="O256" t="n">
         <v>0</v>
       </c>
@@ -39311,7 +39331,11 @@
         <v>0</v>
       </c>
       <c r="V256" t="inlineStr"/>
-      <c r="W256" t="inlineStr"/>
+      <c r="W256" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4354/58518/fa3fc7e3-f637-4843-8df4-9737eb68bd4a.jpg</t>
+        </is>
+      </c>
       <c r="X256" t="n">
         <v>0</v>
       </c>
@@ -39753,7 +39777,11 @@
         <v>148714</v>
       </c>
       <c r="M259" t="inlineStr"/>
-      <c r="N259" t="inlineStr"/>
+      <c r="N259" t="inlineStr">
+        <is>
+          <t>1781975169722</t>
+        </is>
+      </c>
       <c r="O259" t="n">
         <v>0</v>
       </c>
@@ -39774,7 +39802,11 @@
         <v>0</v>
       </c>
       <c r="V259" t="inlineStr"/>
-      <c r="W259" t="inlineStr"/>
+      <c r="W259" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4354/644002/6c305558-b214-496d-9434-63855347395a.jpg</t>
+        </is>
+      </c>
       <c r="X259" t="n">
         <v>0</v>
       </c>
@@ -40051,7 +40083,11 @@
         <v>148716</v>
       </c>
       <c r="M261" t="inlineStr"/>
-      <c r="N261" t="inlineStr"/>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>1781974985915</t>
+        </is>
+      </c>
       <c r="O261" t="n">
         <v>0</v>
       </c>
@@ -40072,7 +40108,11 @@
         <v>0</v>
       </c>
       <c r="V261" t="inlineStr"/>
-      <c r="W261" t="inlineStr"/>
+      <c r="W261" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4354/644004/946de2b1-f305-449e-88ec-03ed0c983c52.jpg</t>
+        </is>
+      </c>
       <c r="X261" t="n">
         <v>0</v>
       </c>
@@ -61074,7 +61114,11 @@
         <v>64733</v>
       </c>
       <c r="M398" t="inlineStr"/>
-      <c r="N398" t="inlineStr"/>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t>1781975346942</t>
+        </is>
+      </c>
       <c r="O398" t="n">
         <v>0</v>
       </c>
@@ -61095,7 +61139,11 @@
         <v>0</v>
       </c>
       <c r="V398" t="inlineStr"/>
-      <c r="W398" t="inlineStr"/>
+      <c r="W398" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4726/64643/49a417c9-faaa-4c0c-bca7-f4831e278e42.jpg</t>
+        </is>
+      </c>
       <c r="X398" t="n">
         <v>0</v>
       </c>
@@ -65904,7 +65952,11 @@
         <v>64759</v>
       </c>
       <c r="M430" t="inlineStr"/>
-      <c r="N430" t="inlineStr"/>
+      <c r="N430" t="inlineStr">
+        <is>
+          <t>1781975166154</t>
+        </is>
+      </c>
       <c r="O430" t="n">
         <v>0</v>
       </c>
@@ -65925,7 +65977,11 @@
         <v>0</v>
       </c>
       <c r="V430" t="inlineStr"/>
-      <c r="W430" t="inlineStr"/>
+      <c r="W430" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4729/64669/cec77346-71f5-4fa9-b3ce-6d6950643853.jpg</t>
+        </is>
+      </c>
       <c r="X430" t="n">
         <v>0</v>
       </c>
@@ -66053,7 +66109,11 @@
         <v>64760</v>
       </c>
       <c r="M431" t="inlineStr"/>
-      <c r="N431" t="inlineStr"/>
+      <c r="N431" t="inlineStr">
+        <is>
+          <t>1781974985005</t>
+        </is>
+      </c>
       <c r="O431" t="n">
         <v>0</v>
       </c>
@@ -66074,7 +66134,11 @@
         <v>0</v>
       </c>
       <c r="V431" t="inlineStr"/>
-      <c r="W431" t="inlineStr"/>
+      <c r="W431" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4729/64670/42cde8e5-f1e0-43a3-804e-1cc558a3f723.jpg</t>
+        </is>
+      </c>
       <c r="X431" t="n">
         <v>0</v>
       </c>
@@ -66202,7 +66266,11 @@
         <v>64761</v>
       </c>
       <c r="M432" t="inlineStr"/>
-      <c r="N432" t="inlineStr"/>
+      <c r="N432" t="inlineStr">
+        <is>
+          <t>1781975165502</t>
+        </is>
+      </c>
       <c r="O432" t="n">
         <v>0</v>
       </c>
@@ -66223,7 +66291,11 @@
         <v>0</v>
       </c>
       <c r="V432" t="inlineStr"/>
-      <c r="W432" t="inlineStr"/>
+      <c r="W432" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4729/64671/c413c988-26a5-459a-a22d-a8ca5f852427.jpg</t>
+        </is>
+      </c>
       <c r="X432" t="n">
         <v>0</v>
       </c>
@@ -66351,7 +66423,11 @@
         <v>64762</v>
       </c>
       <c r="M433" t="inlineStr"/>
-      <c r="N433" t="inlineStr"/>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t>1781975169663</t>
+        </is>
+      </c>
       <c r="O433" t="n">
         <v>0</v>
       </c>
@@ -66372,7 +66448,11 @@
         <v>0</v>
       </c>
       <c r="V433" t="inlineStr"/>
-      <c r="W433" t="inlineStr"/>
+      <c r="W433" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4729/64672/48c4cc56-fda3-49e8-804d-a99d94f5ca51.jpg</t>
+        </is>
+      </c>
       <c r="X433" t="n">
         <v>0</v>
       </c>
@@ -66814,7 +66894,11 @@
         <v>151227</v>
       </c>
       <c r="M436" t="inlineStr"/>
-      <c r="N436" t="inlineStr"/>
+      <c r="N436" t="inlineStr">
+        <is>
+          <t>1781974982952</t>
+        </is>
+      </c>
       <c r="O436" t="n">
         <v>0</v>
       </c>
@@ -66835,7 +66919,11 @@
         <v>0</v>
       </c>
       <c r="V436" t="inlineStr"/>
-      <c r="W436" t="inlineStr"/>
+      <c r="W436" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4729/646514/bb0fa014-b367-41a7-b8f0-dab2c523a540.jpg</t>
+        </is>
+      </c>
       <c r="X436" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 12:29:31
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -2083,7 +2083,11 @@
         <v>58445</v>
       </c>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>1781975706731</t>
+        </is>
+      </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
@@ -2104,7 +2108,11 @@
         <v>0</v>
       </c>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58354/4a7bb637-bbed-47a8-90bb-25d5ff07d793.jpg</t>
+        </is>
+      </c>
       <c r="X11" t="n">
         <v>0</v>
       </c>
@@ -4068,7 +4076,11 @@
         <v>148636</v>
       </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>1781976065172</t>
+        </is>
+      </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
@@ -4089,7 +4101,11 @@
         <v>0</v>
       </c>
       <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/643924/9ec5a52c-b3e0-42c4-862b-6f73b1134c4a.jpg</t>
+        </is>
+      </c>
       <c r="X24" t="n">
         <v>0</v>
       </c>
@@ -4374,7 +4390,11 @@
         <v>58456</v>
       </c>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>1781976245361</t>
+        </is>
+      </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
@@ -4395,7 +4415,11 @@
         <v>0</v>
       </c>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4345/58365/91beeeae-b5ce-439c-95c0-61df79a6bd36.jpg</t>
+        </is>
+      </c>
       <c r="X26" t="n">
         <v>0</v>
       </c>
@@ -4821,7 +4845,11 @@
         <v>58459</v>
       </c>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>1781976425419</t>
+        </is>
+      </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
@@ -4842,7 +4870,11 @@
         <v>0</v>
       </c>
       <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4345/58368/a1f2d7cb-0741-4ae7-9889-7cbc138b33d9.jpg</t>
+        </is>
+      </c>
       <c r="X29" t="n">
         <v>0</v>
       </c>
@@ -23051,7 +23083,11 @@
         <v>58546</v>
       </c>
       <c r="M149" t="inlineStr"/>
-      <c r="N149" t="inlineStr"/>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>1781975531047</t>
+        </is>
+      </c>
       <c r="O149" t="n">
         <v>0</v>
       </c>
@@ -23072,7 +23108,11 @@
         <v>0</v>
       </c>
       <c r="V149" t="inlineStr"/>
-      <c r="W149" t="inlineStr"/>
+      <c r="W149" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4349/58455/7df59ea8-9fc0-416d-ad87-0b4b89b012c7.jpg</t>
+        </is>
+      </c>
       <c r="X149" t="n">
         <v>0</v>
       </c>
@@ -39934,7 +39974,11 @@
         <v>148715</v>
       </c>
       <c r="M260" t="inlineStr"/>
-      <c r="N260" t="inlineStr"/>
+      <c r="N260" t="inlineStr">
+        <is>
+          <t>1781975525039</t>
+        </is>
+      </c>
       <c r="O260" t="n">
         <v>0</v>
       </c>
@@ -39955,7 +39999,11 @@
         <v>0</v>
       </c>
       <c r="V260" t="inlineStr"/>
-      <c r="W260" t="inlineStr"/>
+      <c r="W260" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4354/644003/68ec328b-1bb0-459b-a4e4-0a3855641e30.jpg</t>
+        </is>
+      </c>
       <c r="X260" t="n">
         <v>0</v>
       </c>
@@ -61271,7 +61319,11 @@
         <v>64734</v>
       </c>
       <c r="M399" t="inlineStr"/>
-      <c r="N399" t="inlineStr"/>
+      <c r="N399" t="inlineStr">
+        <is>
+          <t>1781975887400</t>
+        </is>
+      </c>
       <c r="O399" t="n">
         <v>0</v>
       </c>
@@ -61292,7 +61344,11 @@
         <v>0</v>
       </c>
       <c r="V399" t="inlineStr"/>
-      <c r="W399" t="inlineStr"/>
+      <c r="W399" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/412/4726/64644/ae094b1c-861f-466e-94a5-a73591f7351b.jpg</t>
+        </is>
+      </c>
       <c r="X399" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Auto-refresh live election results
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,227 +420,227 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Election ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Election Name</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Election Date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Ward</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Ward Code</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Ward ID</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Polling Unit</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PU Code</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>PU ID</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Polling Unit ID</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Result Updated Time</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Session</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Result Info PU</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Image File</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Image URL</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
@@ -70497,162 +70485,162 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ward</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>
@@ -73793,157 +73781,157 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>
@@ -74162,152 +74150,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>

</xml_diff>

<commit_message>
Refresh INEC feeds and preserve collation
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,227 +432,227 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Election ID</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Election Name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Election Date</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Ward</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Ward Code</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ward ID</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Polling Unit</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PU Code</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>PU ID</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Polling Unit ID</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Result Updated Time</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Session</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Result Info PU</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Image File</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Image URL</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
@@ -706,7 +718,11 @@
         <v>58436</v>
       </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1781981829520</t>
+        </is>
+      </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
@@ -727,7 +743,11 @@
         <v>0</v>
       </c>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58345/ccae3538-0356-4def-bfac-3d8f4675f21a.jpg</t>
+        </is>
+      </c>
       <c r="X2" t="n">
         <v>0</v>
       </c>
@@ -855,7 +875,11 @@
         <v>58437</v>
       </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1781981644306</t>
+        </is>
+      </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
@@ -876,7 +900,11 @@
         <v>0</v>
       </c>
       <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58346/11831b37-ab96-4043-87ba-176bc2b2c5b9.jpg</t>
+        </is>
+      </c>
       <c r="X3" t="n">
         <v>0</v>
       </c>
@@ -1789,7 +1817,11 @@
         <v>58443</v>
       </c>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1781982363781</t>
+        </is>
+      </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
@@ -1810,7 +1842,11 @@
         <v>0</v>
       </c>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58352/36b573c9-a91b-4e8a-b92e-3cf1f8ab63fb.jpg</t>
+        </is>
+      </c>
       <c r="X9" t="n">
         <v>0</v>
       </c>
@@ -1938,7 +1974,11 @@
         <v>58444</v>
       </c>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1781983756086</t>
+        </is>
+      </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
@@ -1959,7 +1999,11 @@
         <v>0</v>
       </c>
       <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58353/454f77e5-8f35-4017-b9c0-9c3e4a43c7a0.jpg</t>
+        </is>
+      </c>
       <c r="X10" t="n">
         <v>0</v>
       </c>
@@ -3335,7 +3379,11 @@
         <v>58453</v>
       </c>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>1781981828728</t>
+        </is>
+      </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
@@ -3356,7 +3404,11 @@
         <v>0</v>
       </c>
       <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58362/4c9d3e63-95fe-4496-a881-82ca209ffba5.jpg</t>
+        </is>
+      </c>
       <c r="X19" t="n">
         <v>0</v>
       </c>
@@ -3484,7 +3536,11 @@
         <v>58454</v>
       </c>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>1781981469293</t>
+        </is>
+      </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
@@ -3505,7 +3561,11 @@
         <v>0</v>
       </c>
       <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4344/58363/aaa83413-d111-4fa5-9620-e70bc4a72dc6.jpg</t>
+        </is>
+      </c>
       <c r="X20" t="n">
         <v>0</v>
       </c>
@@ -19792,7 +19852,11 @@
         <v>58526</v>
       </c>
       <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>1781981105891</t>
+        </is>
+      </c>
       <c r="O124" t="n">
         <v>0</v>
       </c>
@@ -19813,7 +19877,11 @@
         <v>0</v>
       </c>
       <c r="V124" t="inlineStr"/>
-      <c r="W124" t="inlineStr"/>
+      <c r="W124" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4348/58435/98b69f77-a004-43ca-9707-405d64d038ad.jpg</t>
+        </is>
+      </c>
       <c r="X124" t="n">
         <v>0</v>
       </c>
@@ -23370,29 +23438,43 @@
       <c r="L147" t="n">
         <v>58544</v>
       </c>
-      <c r="M147" t="inlineStr"/>
-      <c r="N147" t="inlineStr"/>
+      <c r="M147" t="n">
+        <v>1781981468267</v>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>1781981467671</t>
+        </is>
+      </c>
       <c r="O147" t="n">
-        <v>0</v>
+        <v>997</v>
       </c>
       <c r="P147" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="Q147" t="n">
         <v>0</v>
       </c>
-      <c r="R147" t="inlineStr"/>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>6a36e11bc89f29392f333c6e</t>
+        </is>
+      </c>
       <c r="S147" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="T147" t="n">
-        <v>0</v>
+        <v>997</v>
       </c>
       <c r="U147" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="V147" t="inlineStr"/>
-      <c r="W147" t="inlineStr"/>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4349/58453/5f092f32-c2c4-4146-a609-a53268787a8e.jpg</t>
+        </is>
+      </c>
       <c r="X147" t="n">
         <v>0</v>
       </c>
@@ -23409,7 +23491,7 @@
         <v>0</v>
       </c>
       <c r="AC147" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="AD147" t="n">
         <v>0</v>
@@ -23834,7 +23916,11 @@
         <v>58547</v>
       </c>
       <c r="M150" t="inlineStr"/>
-      <c r="N150" t="inlineStr"/>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>1781981467380</t>
+        </is>
+      </c>
       <c r="O150" t="n">
         <v>0</v>
       </c>
@@ -23855,7 +23941,11 @@
         <v>0</v>
       </c>
       <c r="V150" t="inlineStr"/>
-      <c r="W150" t="inlineStr"/>
+      <c r="W150" t="inlineStr">
+        <is>
+          <t>https://inc-s3-cache.incportals.com/cached/express/results/2992/20/378/4349/58456/c835662b-bbe8-4286-9256-cbc3c23c9eab.jpg</t>
+        </is>
+      </c>
       <c r="X150" t="n">
         <v>0</v>
       </c>
@@ -70481,168 +70571,178 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF31"/>
+  <dimension ref="A1:AH31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ward</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>INEC Uploaded Results</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>INEC Upload Percent</t>
         </is>
       </c>
     </row>
@@ -70749,6 +70849,12 @@
       <c r="AF2" t="n">
         <v>23</v>
       </c>
+      <c r="AG2" t="n">
+        <v>22</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>95.7</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -70853,6 +70959,12 @@
       <c r="AF3" t="n">
         <v>17</v>
       </c>
+      <c r="AG3" t="n">
+        <v>17</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -70957,6 +71069,12 @@
       <c r="AF4" t="n">
         <v>44</v>
       </c>
+      <c r="AG4" t="n">
+        <v>44</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -71061,6 +71179,12 @@
       <c r="AF5" t="n">
         <v>27</v>
       </c>
+      <c r="AG5" t="n">
+        <v>27</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -71165,6 +71289,12 @@
       <c r="AF6" t="n">
         <v>21</v>
       </c>
+      <c r="AG6" t="n">
+        <v>15</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>71.40000000000001</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -71183,22 +71313,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>997</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>997</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -71216,7 +71346,7 @@
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
@@ -71268,6 +71398,12 @@
       </c>
       <c r="AF7" t="n">
         <v>24</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>23</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>95.8</v>
       </c>
     </row>
     <row r="8">
@@ -71373,6 +71509,12 @@
       <c r="AF8" t="n">
         <v>13</v>
       </c>
+      <c r="AG8" t="n">
+        <v>13</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -71477,6 +71619,12 @@
       <c r="AF9" t="n">
         <v>12</v>
       </c>
+      <c r="AG9" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>83.3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -71581,6 +71729,12 @@
       <c r="AF10" t="n">
         <v>35</v>
       </c>
+      <c r="AG10" t="n">
+        <v>34</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>97.09999999999999</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -71685,6 +71839,12 @@
       <c r="AF11" t="n">
         <v>34</v>
       </c>
+      <c r="AG11" t="n">
+        <v>33</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>97.09999999999999</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -71789,6 +71949,12 @@
       <c r="AF12" t="n">
         <v>10</v>
       </c>
+      <c r="AG12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -71893,6 +72059,12 @@
       <c r="AF13" t="n">
         <v>11</v>
       </c>
+      <c r="AG13" t="n">
+        <v>7</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>63.6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -71997,6 +72169,12 @@
       <c r="AF14" t="n">
         <v>10</v>
       </c>
+      <c r="AG14" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -72101,6 +72279,12 @@
       <c r="AF15" t="n">
         <v>14</v>
       </c>
+      <c r="AG15" t="n">
+        <v>14</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -72205,6 +72389,12 @@
       <c r="AF16" t="n">
         <v>8</v>
       </c>
+      <c r="AG16" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -72309,6 +72499,12 @@
       <c r="AF17" t="n">
         <v>5</v>
       </c>
+      <c r="AG17" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -72413,6 +72609,12 @@
       <c r="AF18" t="n">
         <v>7</v>
       </c>
+      <c r="AG18" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>85.7</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -72517,6 +72719,12 @@
       <c r="AF19" t="n">
         <v>9</v>
       </c>
+      <c r="AG19" t="n">
+        <v>9</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -72621,6 +72829,12 @@
       <c r="AF20" t="n">
         <v>7</v>
       </c>
+      <c r="AG20" t="n">
+        <v>7</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -72725,6 +72939,12 @@
       <c r="AF21" t="n">
         <v>9</v>
       </c>
+      <c r="AG21" t="n">
+        <v>9</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -72829,6 +73049,12 @@
       <c r="AF22" t="n">
         <v>12</v>
       </c>
+      <c r="AG22" t="n">
+        <v>12</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -72933,6 +73159,12 @@
       <c r="AF23" t="n">
         <v>11</v>
       </c>
+      <c r="AG23" t="n">
+        <v>11</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -73037,6 +73269,12 @@
       <c r="AF24" t="n">
         <v>9</v>
       </c>
+      <c r="AG24" t="n">
+        <v>9</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -73141,6 +73379,12 @@
       <c r="AF25" t="n">
         <v>11</v>
       </c>
+      <c r="AG25" t="n">
+        <v>11</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -73245,6 +73489,12 @@
       <c r="AF26" t="n">
         <v>10</v>
       </c>
+      <c r="AG26" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -73349,6 +73599,12 @@
       <c r="AF27" t="n">
         <v>11</v>
       </c>
+      <c r="AG27" t="n">
+        <v>9</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>81.8</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -73453,6 +73709,12 @@
       <c r="AF28" t="n">
         <v>15</v>
       </c>
+      <c r="AG28" t="n">
+        <v>14</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>93.3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -73557,6 +73819,12 @@
       <c r="AF29" t="n">
         <v>9</v>
       </c>
+      <c r="AG29" t="n">
+        <v>9</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -73661,6 +73929,12 @@
       <c r="AF30" t="n">
         <v>8</v>
       </c>
+      <c r="AG30" t="n">
+        <v>8</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -73764,6 +74038,12 @@
       </c>
       <c r="AF31" t="n">
         <v>10</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -73777,163 +74057,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>INEC Uploaded Results</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>INEC Upload Percent</t>
         </is>
       </c>
     </row>
@@ -73949,22 +74239,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3183</v>
+        <v>4180</v>
       </c>
       <c r="D2" t="n">
-        <v>390</v>
+        <v>468</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>390</v>
+        <v>452</v>
       </c>
       <c r="G2" t="n">
-        <v>3183</v>
+        <v>4180</v>
       </c>
       <c r="H2" t="n">
-        <v>388</v>
+        <v>450</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -73982,7 +74272,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>384</v>
+        <v>446</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -74034,6 +74324,12 @@
       </c>
       <c r="AE2" t="n">
         <v>303</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>283</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -74133,6 +74429,12 @@
       </c>
       <c r="AE3" t="n">
         <v>143</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>139</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>97.2</v>
       </c>
     </row>
   </sheetData>
@@ -74146,158 +74448,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>INEC Uploaded Results</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>INEC Expected Results</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>INEC Upload Percent</t>
         </is>
       </c>
     </row>
@@ -74308,22 +74625,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6314</v>
+        <v>7311</v>
       </c>
       <c r="C2" t="n">
-        <v>906</v>
+        <v>984</v>
       </c>
       <c r="D2" t="n">
         <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>903</v>
+        <v>965</v>
       </c>
       <c r="F2" t="n">
-        <v>6272</v>
+        <v>7269</v>
       </c>
       <c r="G2" t="n">
-        <v>896</v>
+        <v>958</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -74341,7 +74658,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>887</v>
+        <v>949</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -74393,6 +74710,15 @@
       </c>
       <c r="AD2" t="n">
         <v>446</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>422</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>446</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>94.59999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-20 17:14:14
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,227 +432,227 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Election ID</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Election Name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Election Date</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Ward</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Ward Code</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ward ID</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Polling Unit</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PU Code</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>PU ID</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Polling Unit ID</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Result Updated Time</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Session</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Result Info PU</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Image File</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Image URL</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
@@ -70627,172 +70639,172 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ward</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>INEC Uploaded Results</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>INEC Upload Percent</t>
         </is>
@@ -74113,167 +74125,167 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>INEC Uploaded Results</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>INEC Upload Percent</t>
         </is>
@@ -74504,167 +74516,167 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>INEC Uploaded Results</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>INEC Expected Results</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>INEC Upload Percent</t>
         </is>

</xml_diff>

<commit_message>
Auto-refresh live election results 2026-06-21 12:58:48
</commit_message>
<xml_diff>
--- a/output/Kano/results.xlsx
+++ b/output/Kano/results.xlsx
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,227 +432,227 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Election ID</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Election Name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Election Date</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Ward</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Ward Code</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ward ID</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Polling Unit</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PU Code</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>PU ID</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Polling Unit ID</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Result Updated Time</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Session</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Result Info PU</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Image File</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Image URL</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
@@ -70627,172 +70639,172 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ward</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>INEC Uploaded Results</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>INEC Upload Percent</t>
         </is>
@@ -74113,167 +74125,167 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LGA</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>INEC Uploaded Results</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>INEC Upload Percent</t>
         </is>
@@ -74504,167 +74516,167 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ballots Issued</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ballots Used</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Invalid Votes</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Total Accredited</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total Registered</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Valid Votes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>AAC</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ADC</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ADP</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>APC</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>APGA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>APM</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>APP</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>BP</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>DLA</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>LP</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>NDC</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>NDP</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>NNPP</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>NRM</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>PDP</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>SDP</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>YP</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>YPP</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>ZLP</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Polling Units</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>INEC Uploaded Results</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>INEC Expected Results</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>INEC Upload Percent</t>
         </is>

</xml_diff>